<commit_message>
Correccion error en celda de version
</commit_message>
<xml_diff>
--- a/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_CPU.xlsx
+++ b/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_CPU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reozen/Team Dropbox/David Garrido/MUSOTOKU/PROJECTS/BATTERYPACK - FALCON/00.REPOSITORIES/BATTERY-PACK/02.HARDWARE/V2-ROVER R-1/02.BOM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\02.HARDWARE\V2-ROVER R-1\02.BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F865C664-9C96-D04B-9290-CCF6BB2B1EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DDF985-E6F1-4004-9A77-A32E2386CFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="19420" windowHeight="26580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BATT_CPU" sheetId="1" r:id="rId1"/>
@@ -1150,49 +1150,49 @@
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Hipervínculo" xfId="42" builtinId="8"/>
+    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -1305,9 +1305,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1345,7 +1345,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1451,7 +1451,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1593,7 +1593,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1602,24 +1602,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="122.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="122.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -1629,14 +1629,14 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="27" x14ac:dyDescent="0.4">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5"/>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:8" ht="26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="27" x14ac:dyDescent="0.4">
       <c r="C4" s="23" t="s">
         <v>22</v>
       </c>
@@ -1644,13 +1644,13 @@
       <c r="E4" s="24"/>
       <c r="F4" s="25"/>
     </row>
-    <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C5" s="6"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>8</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>11</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>12</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>13</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>14</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>15</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>16</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>17</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>18</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>19</v>
       </c>
@@ -2116,7 +2116,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>20</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>21</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>22</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>23</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>24</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>25</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>26</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>27</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>28</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>29</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>30</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>31</v>
       </c>
@@ -2447,17 +2447,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15976B5A-CF8E-C940-9265-A2311480139B}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="135.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="135.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>69</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -2513,7 +2513,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -2555,7 +2555,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
@@ -2597,7 +2597,10 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>9</v>
+      </c>
       <c r="B13" s="22">
         <v>45195</v>
       </c>
@@ -2616,56 +2619,56 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7076B1D4-2B71-F94B-B48B-67B36DACA7AE}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
         <v>77</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
     </row>
-    <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>78</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="16"/>
     </row>
-    <row r="3" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>79</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="16"/>
     </row>
-    <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <v>28805</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
     </row>
-    <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>80</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="16"/>
     </row>
-    <row r="6" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>81</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
     </row>
-    <row r="7" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
     </row>
-    <row r="8" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>82</v>
       </c>
@@ -2674,7 +2677,7 @@
       </c>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
Revert "Merge pull request #84 from MSTKMAD/develop"
This reverts commit 96fc117d3460fb5d771273194348358b85af1598, reversing
changes made to 9bb4215ab554844daf6eea25f914757804df500a.
</commit_message>
<xml_diff>
--- a/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_CPU.xlsx
+++ b/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_CPU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\02.HARDWARE\V2-ROVER R-1\02.BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reozen/Team Dropbox/David Garrido/MUSOTOKU/PROJECTS/BATTERYPACK - FALCON/00.REPOSITORIES/BATTERY-PACK/02.HARDWARE/V2-ROVER R-1/02.BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93DDF985-E6F1-4004-9A77-A32E2386CFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F865C664-9C96-D04B-9290-CCF6BB2B1EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="19420" windowHeight="26580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BATT_CPU" sheetId="1" r:id="rId1"/>
@@ -1150,49 +1150,49 @@
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Hipervínculo" xfId="42" builtinId="8"/>
-    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -1305,9 +1305,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1345,7 +1345,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1451,7 +1451,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1593,7 +1593,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1602,24 +1602,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="122.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="122.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -1629,14 +1629,14 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="27" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="26" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5"/>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:8" ht="27" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="26" x14ac:dyDescent="0.25">
       <c r="C4" s="23" t="s">
         <v>22</v>
       </c>
@@ -1644,13 +1644,13 @@
       <c r="E4" s="24"/>
       <c r="F4" s="25"/>
     </row>
-    <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="6"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>5</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>6</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>7</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>8</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>11</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>12</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>13</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>14</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>15</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>16</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>17</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>18</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>19</v>
       </c>
@@ -2116,7 +2116,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>20</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>21</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>22</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>23</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>24</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>25</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>26</v>
       </c>
@@ -2289,7 +2289,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>27</v>
       </c>
@@ -2315,7 +2315,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>28</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>29</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>30</v>
       </c>
@@ -2387,7 +2387,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>31</v>
       </c>
@@ -2447,17 +2447,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15976B5A-CF8E-C940-9265-A2311480139B}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="135.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="135.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>69</v>
       </c>
@@ -2471,7 +2471,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -2513,7 +2513,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>4</v>
       </c>
@@ -2527,7 +2527,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>5</v>
       </c>
@@ -2541,7 +2541,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>6</v>
       </c>
@@ -2555,7 +2555,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="64" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>7</v>
       </c>
@@ -2569,7 +2569,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>8</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9</v>
       </c>
@@ -2597,10 +2597,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>9</v>
-      </c>
+    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="B13" s="22">
         <v>45195</v>
       </c>
@@ -2619,56 +2616,56 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7076B1D4-2B71-F94B-B48B-67B36DACA7AE}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
         <v>77</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
     </row>
-    <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
         <v>78</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="16"/>
     </row>
-    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
         <v>79</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="16"/>
     </row>
-    <row r="4" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A4" s="15">
         <v>28805</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
     </row>
-    <row r="5" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>80</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="16"/>
     </row>
-    <row r="6" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
         <v>81</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
     </row>
-    <row r="7" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
     </row>
-    <row r="8" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A8" s="17" t="s">
         <v>82</v>
       </c>
@@ -2677,7 +2674,7 @@
       </c>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="19" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
Salto del compardor en arranques de alguna maquinas. #86
</commit_message>
<xml_diff>
--- a/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_CPU.xlsx
+++ b/02.HARDWARE/V2-ROVER R-1/02.BOM/BATT_CPU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reozen/Team Dropbox/David Garrido/MUSOTOKU/PROJECTS/BATTERYPACK - FALCON/00.REPOSITORIES/BATTERY-PACK/02.HARDWARE/V2-ROVER R-1/02.BOM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Team Dropbox\JRODRIGUEZ\Repositorios\01.Rover\02.HARDWARE\V2-ROVER R-1\02.BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F865C664-9C96-D04B-9290-CCF6BB2B1EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E156BA56-A77C-43E0-8B3A-450F2E8F7127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="19420" windowHeight="26580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BATT_CPU" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="125">
   <si>
     <t>Qty</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>R11</t>
-  </si>
-  <si>
-    <t>8k2</t>
   </si>
   <si>
     <t>U3</t>
@@ -412,6 +409,12 @@
   </si>
   <si>
     <t>Se actualiza la columna de NEW para que SETI tenga los cambios actualizados contra la version anterior (7)</t>
+  </si>
+  <si>
+    <t>11k</t>
+  </si>
+  <si>
+    <t>Se cambia el valor de R11 de 8k2 a 11k.</t>
   </si>
 </sst>
 </file>
@@ -1084,7 +1087,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1148,51 +1151,52 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Énfasis6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Énfasis6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Énfasis6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Bueno" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Celda de comprobación" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Celda vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Encabezado 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Encabezado 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Énfasis1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Énfasis2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Énfasis3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Énfasis4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Hipervínculo" xfId="42" builtinId="8"/>
+    <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -1305,9 +1309,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1345,7 +1349,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1451,7 +1455,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1593,7 +1597,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1602,66 +1606,66 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="122.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="122.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="3">
         <f>MAX(_HISTORY!A4:A43)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="26" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="27" x14ac:dyDescent="0.4">
       <c r="A3" s="4"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5"/>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:8" ht="26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="27" x14ac:dyDescent="0.4">
       <c r="C4" s="23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D4" s="24"/>
       <c r="E4" s="24"/>
       <c r="F4" s="25"/>
     </row>
-    <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C5" s="6"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>1</v>
@@ -1673,254 +1677,254 @@
         <v>3</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C8" s="1">
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C9" s="1">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C10" s="1">
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C11" s="1">
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C12" s="1">
         <v>18</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C13" s="1">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="1">
         <v>3</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G14" t="s">
         <v>6</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" s="1">
         <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E15" t="s">
         <v>5</v>
       </c>
       <c r="F15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G15" t="s">
         <v>6</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" s="1">
         <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
         <v>15</v>
       </c>
-      <c r="G16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
@@ -1929,16 +1933,16 @@
         <v>7</v>
       </c>
       <c r="E17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
         <v>15</v>
       </c>
-      <c r="G17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>12</v>
       </c>
@@ -1952,462 +1956,462 @@
         <v>8</v>
       </c>
       <c r="E18" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
         <v>15</v>
       </c>
-      <c r="G18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C19" s="1">
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
         <v>15</v>
       </c>
-      <c r="G19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" s="1">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
         <v>15</v>
       </c>
-      <c r="G20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C21" s="1">
         <v>4</v>
       </c>
       <c r="D21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E21" t="s">
         <v>4</v>
       </c>
       <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
         <v>15</v>
       </c>
-      <c r="G21" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C22" s="1">
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
         <v>15</v>
       </c>
-      <c r="G22" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C23" s="1">
         <v>0</v>
       </c>
       <c r="D23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E23" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C24" s="1">
         <v>3</v>
       </c>
       <c r="D24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
         <v>15</v>
       </c>
-      <c r="G24" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" s="1">
         <v>3</v>
       </c>
       <c r="D25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
         <v>15</v>
       </c>
-      <c r="G25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>20</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C26" s="1">
         <v>3</v>
       </c>
       <c r="D26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C27" s="1">
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G27" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>22</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28" s="1">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G28" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>23</v>
       </c>
       <c r="B29" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" s="1">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G29" t="s">
+        <v>98</v>
+      </c>
+      <c r="H29" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="H29" s="12" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>24</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C31" s="1">
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E31" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F31" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F31" s="10" t="s">
-        <v>67</v>
-      </c>
       <c r="G31" s="10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C32" s="1">
         <v>1</v>
       </c>
       <c r="D32" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E32" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>27</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C33" s="21">
         <v>0</v>
       </c>
       <c r="D33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H33" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>28</v>
       </c>
       <c r="B34" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C34" s="21">
         <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E34" t="s">
+        <v>110</v>
+      </c>
+      <c r="F34" t="s">
+        <v>20</v>
+      </c>
+      <c r="G34" t="s">
+        <v>16</v>
+      </c>
+      <c r="H34" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="F34" t="s">
-        <v>21</v>
-      </c>
-      <c r="G34" t="s">
-        <v>17</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>29</v>
       </c>
       <c r="B35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C35" s="21">
         <v>1</v>
       </c>
       <c r="D35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E35" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
         <v>15</v>
       </c>
-      <c r="G35" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>30</v>
       </c>
       <c r="B36" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C36" s="21">
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
         <v>15</v>
       </c>
-      <c r="G36" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>31</v>
       </c>
       <c r="B37" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C37" s="21">
         <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
         <v>15</v>
-      </c>
-      <c r="G37" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -2446,32 +2450,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15976B5A-CF8E-C940-9265-A2311480139B}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="135.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="135.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="B3" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2479,13 +2483,13 @@
         <v>44874</v>
       </c>
       <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="s">
         <v>73</v>
       </c>
-      <c r="D4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -2493,13 +2497,13 @@
         <v>44880</v>
       </c>
       <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
         <v>75</v>
       </c>
-      <c r="D5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -2507,13 +2511,13 @@
         <v>44918</v>
       </c>
       <c r="C6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -2521,13 +2525,13 @@
         <v>44931</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -2535,13 +2539,13 @@
         <v>44958</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -2549,13 +2553,13 @@
         <v>45062</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -2563,13 +2567,13 @@
         <v>45063</v>
       </c>
       <c r="C10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
@@ -2577,13 +2581,13 @@
         <v>45180</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
@@ -2591,21 +2595,35 @@
         <v>45194</v>
       </c>
       <c r="C12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" s="22">
         <v>45195</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" s="27">
+        <v>45540</v>
+      </c>
+      <c r="C14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2616,70 +2634,70 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7076B1D4-2B71-F94B-B48B-67B36DACA7AE}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
     </row>
-    <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="16"/>
     </row>
-    <row r="3" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="16"/>
     </row>
-    <row r="4" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <v>28805</v>
       </c>
       <c r="B4" s="16"/>
       <c r="C4" s="16"/>
     </row>
-    <row r="5" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="16"/>
     </row>
-    <row r="6" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
     </row>
-    <row r="7" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="B7" s="16"/>
       <c r="C7" s="16"/>
     </row>
-    <row r="8" spans="1:3" ht="19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="19"/>
+    </row>
+    <row r="9" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C8" s="19"/>
-    </row>
-    <row r="9" spans="1:3" ht="19" x14ac:dyDescent="0.2">
-      <c r="A9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>84</v>
-      </c>
-      <c r="B9" s="16" t="s">
-        <v>85</v>
       </c>
       <c r="C9" s="16"/>
     </row>

</xml_diff>